<commit_message>
Training 25/26 kits intentional; kit part wording not a shirt/kit error
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149ELLgZdjaY7wRsdGLp26m
</commit_message>
<xml_diff>
--- a/listing-monitor/reports/2026-10-29/qa_2026-10-29.xlsx
+++ b/listing-monitor/reports/2026-10-29/qa_2026-10-29.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cần xác nhận" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'KFK'!$A$1:$N$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CFS'!$A$1:$N$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'KFK'!$A$1:$N$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CFS'!$A$1:$N$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tạo lúc 2026-10-29 23:33. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
+          <t>Tạo lúc 2026-10-30 06:55. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
         <v>14</v>
@@ -565,7 +565,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G6" t="n">
         <v>31</v>
@@ -654,14 +654,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sai loại Shirt/Kit</t>
+          <t>Sai season</t>
         </is>
       </c>
       <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
         <v>3</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>3</v>
@@ -670,192 +670,113 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sai season</t>
+          <t>Sai đối tượng</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sai đối tượng</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D18" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Sai cầu thủ</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Sai cầu thủ</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
         <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Lỗi lặp lại trên phần lớn listing của 1 site (nhiều khả năng do TEMPLATE, sửa template 1 lần)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Nhóm</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Vị trí</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Lỗi</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Số listing</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>CFS</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>16/27</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -869,7 +790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1026,46 +947,46 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>265823</v>
+        <v>265840</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sai loại Shirt/Kit</t>
+          <t>Khuyến mãi Free Pin (KFK)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Trang sản phẩm</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Listing là KIT nhưng description dùng chữ 'shirt' 2 lần: ...t included. What’s Included Long sleeve shirt with Messi name and number 10 already a...</t>
+          <t>Sản phẩm Argentina (1 trong 7 đội có Free Pin) nhưng trang không có chữ 'FREE ARGENTINA PIN'</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Master File 4: kit không ghi 'shirt' và ngược lại</t>
+          <t>Kiểm tra BOGO coupon buy-argentina-get-pin có gồm sản phẩm này không</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -1084,46 +1005,46 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 09:12</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>265840</v>
+        <v>265852</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>KFK_ARG_AWLV_KD_No_1994</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Khuyến mãi Free Pin (KFK)</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Trang sản phẩm</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Sản phẩm Argentina (1 trong 7 đội có Free Pin) nhưng trang không có chữ 'FREE ARGENTINA PIN'</t>
+          <t>1/5 ảnh không có alt text</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra BOGO coupon buy-argentina-get-pin có gồm sản phẩm này không</t>
+          <t>Thêm alt text riêng cho từng ảnh</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -1142,46 +1063,46 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 09:12</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>265840</v>
+        <v>265852</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>KFK_ARG_AWLV_KD_No_1994</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sai loại Shirt/Kit</t>
+          <t>Khuyến mãi Free Pin (KFK)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Trang sản phẩm</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Listing là KIT nhưng description dùng chữ 'shirt' 1 lần: ...t included. What’s Included Long sleeve shirt with Maradona name and number 10 alread...</t>
+          <t>Sản phẩm Argentina (1 trong 7 đội có Free Pin) nhưng trang không có chữ 'FREE ARGENTINA PIN'</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Master File 4: kit không ghi 'shirt' và ngược lại</t>
+          <t>Kiểm tra BOGO coupon buy-argentina-get-pin có gồm sản phẩm này không</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -1200,46 +1121,46 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-29 09:12</t>
+          <t>2026-10-29 15:34</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>265852</v>
+        <v>265903</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_No_1994</t>
+          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 (No Socks, Long Sleeve)</t>
+          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Alt text</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>1/5 ảnh không có alt text</t>
+          <t>'Badge' (...p to 13 letters and 2 digits. Badge options: Premier League sleev...)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Thêm alt text riêng cho từng ảnh</t>
+          <t>Badge -&gt; chest detail</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -1258,46 +1179,46 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-29 09:12</t>
+          <t>2026-10-29 15:48</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>265852</v>
+        <v>265918</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_No_1994</t>
+          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 (No Socks, Long Sleeve)</t>
+          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Khuyến mãi Free Pin (KFK)</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Trang sản phẩm</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Sản phẩm Argentina (1 trong 7 đội có Free Pin) nhưng trang không có chữ 'FREE ARGENTINA PIN'</t>
+          <t>'badge' (...to 2 digits. Adult’s Home kit badge options: Premier League sleev...)</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra BOGO coupon buy-argentina-get-pin có gồm sản phẩm này không</t>
+          <t>badge -&gt; chest detail</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -1316,46 +1237,46 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-29 15:34</t>
+          <t>2026-10-29 15:48</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>265903</v>
+        <v>265918</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
+          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
+          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>'Badge' (...p to 13 letters and 2 digits. Badge options: Premier League sleev...)</t>
+          <t>1/7 ảnh không có alt text</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Badge -&gt; chest detail</t>
+          <t>Thêm alt text riêng cho từng ảnh</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -1374,46 +1295,46 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-29 15:34</t>
+          <t>2026-10-29 15:48</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>265903</v>
+        <v>265918</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
+          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
+          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sai loại Shirt/Kit</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>SKU variation</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Listing là KIT nhưng description dùng chữ 'shirt' 1 lần: ... Options You Can Add Name &amp; number: The shirt is supplied without a name or number. A...</t>
+          <t>SKU cha KFK_CH_HO/AWGP_ADK_No_26/27 nhưng variation mang SKU khác đầu: KFK_CH_AW/HOGP_ADK_No_26/27_S (+4)</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Master File 4: kit không ghi 'shirt' và ngược lại</t>
+          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1425,53 +1346,53 @@
       <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-29 15:48</t>
+          <t>2026-10-29 08:35</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>265918</v>
+        <v>265823</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
+          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>'badge' (...to 2 digits. Adult’s Home kit badge options: Premier League sleev...)</t>
+          <t>SEO title dài 70 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>badge -&gt; chest detail</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1483,53 +1404,53 @@
       <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-29 15:48</t>
+          <t>2026-10-29 08:35</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>265918</v>
+        <v>265823</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
+          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Alt text</t>
+          <t>Meta description</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>1/7 ảnh không có alt text</t>
+          <t>Meta dài 169 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Thêm alt text riêng cho từng ảnh</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1541,53 +1462,53 @@
       <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-29 15:48</t>
+          <t>2026-10-29 08:35</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>265918</v>
+        <v>265823</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
+          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SKU variation</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>SKU cha KFK_CH_HO/AWGP_ADK_No_26/27 nhưng variation mang SKU khác đầu: KFK_CH_AW/HOGP_ADK_No_26/27_S (+4)</t>
+          <t>Alt text bị trùng giữa các ảnh: "Argentina Away Kids Kit 1994-MARADONA 10-over view-long sleeve-no socks"</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
+          <t>Mỗi ảnh 1 alt riêng</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1624,22 +1545,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 70 ký tự (nên &lt;= 60)</t>
+          <t>SKU 'KFK_ARG_AWLV_KD_MESSI 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1664,46 +1585,46 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>265823</v>
+        <v>265834</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Sai cầu thủ</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Meta description</t>
+          <t>Tên sản phẩm</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 169 ký tự (nên &lt;= 160)</t>
+          <t>Tên + số cầu thủ chưa VIẾT HOA</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Viết hoa tên + số cầu thủ</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1722,46 +1643,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>265823</v>
+        <v>265834</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Alt text</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Alt text bị trùng giữa các ảnh: "Argentina Away Kids Kit 1994-MARADONA 10-over view-long sleeve-no socks"</t>
+          <t>SEO title dài 66 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Mỗi ảnh 1 alt riêng</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -1780,46 +1701,46 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>265823</v>
+        <v>265834</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>SKU 'KFK_ARG_AWLV_KD_MESSI 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Alt text bị trùng giữa các ảnh: "Inter Milan Home kids kit 2009_10-IBRAHIMOVIĆ 8-back view-no socks"</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Mỗi ảnh 1 alt riêng</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -1856,22 +1777,22 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sai cầu thủ</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Tên sản phẩm</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Tên + số cầu thủ chưa VIẾT HOA</t>
+          <t>SKU 'KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Viết hoa tên + số cầu thủ</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1900,16 +1821,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>265834</v>
+        <v>265840</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
+          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1924,7 +1845,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 66 ký tự (nên &lt;= 60)</t>
+          <t>SEO title dài 73 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1935,7 +1856,7 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1958,42 +1879,42 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>265834</v>
+        <v>265840</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
+          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Alt text</t>
+          <t>Meta description</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Alt text bị trùng giữa các ảnh: "Inter Milan Home kids kit 2009_10-IBRAHIMOVIĆ 8-back view-no socks"</t>
+          <t>Meta dài 172 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Mỗi ảnh 1 alt riêng</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -2016,16 +1937,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>265834</v>
+        <v>265840</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
+          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2040,7 +1961,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>SKU 'KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SKU 'KFK_ARG_AWLV_KD_MARADONA 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -2051,7 +1972,7 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -2070,20 +1991,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 15:34</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>265840</v>
+        <v>265903</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
+          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2098,7 +2019,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 73 ký tự (nên &lt;= 60)</t>
+          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -2109,7 +2030,7 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2128,46 +2049,46 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 15:34</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>265840</v>
+        <v>265903</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
+          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Meta description</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 172 ký tự (nên &lt;= 160)</t>
+          <t>Chelsea (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2186,46 +2107,46 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 15:48</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>265840</v>
+        <v>265918</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
+          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>SKU 'KFK_ARG_AWLV_KD_MARADONA 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Chelsea (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2236,182 +2157,8 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026-10-29 15:34</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>265903</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>SEO title</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>Rút gọn</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
-        </is>
-      </c>
-      <c r="L24" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2026-10-29 15:34</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>265903</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Club bị report</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Chelsea (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>Check blur logo</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
-        </is>
-      </c>
-      <c r="L25" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026-10-29 15:48</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>265918</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Club bị report</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Chelsea (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>Check blur logo</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
-        </is>
-      </c>
-      <c r="L26" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N26"/>
+  <autoFilter ref="A1:N23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -2457,12 +2204,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2474,7 +2215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3088,53 +2829,53 @@
       <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-29 01:43</t>
+          <t>2026-10-29 14:45</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>85240</v>
+        <v>85544</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CFS_MC_HOLV_KD_No_26/27</t>
+          <t>CFS_RM_HO_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Manchester City Home Kids Cheap Football Kit 2026/27 Long Sleeve</t>
+          <t>Real Madrid Home Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Sai season</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Tên sản phẩm</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Manchester City (Puma): sheet ghi CFS 'Published (blurred PUMA logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/manchester-city-home-kids-cheap-football-kit-2026-27-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-home-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -3153,46 +2894,46 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-29 02:00</t>
+          <t>2026-10-29 01:43</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>85273</v>
+        <v>85240</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CFS_SHW_AW_KD_No_26/27</t>
+          <t>CFS_MC_HOLV_KD_No_26/27</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sheffield Wednesday Away Kids Cheap Football Kit 2026/27</t>
+          <t>Manchester City Home Kids Cheap Football Kit 2026/27 Long Sleeve</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Không xác định được đội/CLB từ tên sản phẩm → cần người check option badge.</t>
+          <t>Manchester City (Puma): sheet ghi CFS 'Published (blurred PUMA logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/sheffield-wednesday-away-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/manchester-city-home-kids-cheap-football-kit-2026-27-long-sleeve/</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -3211,20 +2952,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-29 02:06</t>
+          <t>2026-10-29 02:00</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>85284</v>
+        <v>85273</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CFS_SAFC_GreenGK_KD_No_26/27</t>
+          <t>CFS_SHW_AW_KD_No_26/27</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sunderland AFC Green Goalkeeper Kids Cheap Football Kit 2026/27</t>
+          <t>Sheffield Wednesday Away Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -3239,7 +2980,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu Sunderland đá giải nào mùa 2026/27 → cần người check option badge.</t>
+          <t>Không xác định được đội/CLB từ tên sản phẩm → cần người check option badge.</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -3250,7 +2991,7 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/sunderland-afc-green-goalkeeper-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/sheffield-wednesday-away-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -3269,20 +3010,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-29 02:29</t>
+          <t>2026-10-29 02:06</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>85295</v>
+        <v>85284</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CFS_SAFC_OrangeGK_KD_No_26/27</t>
+          <t>CFS_SAFC_GreenGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sunderland AFC Orange Goalkeeper Kids Cheap Football Kit 2026/27</t>
+          <t>Sunderland AFC Green Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3308,7 +3049,7 @@
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/sunderland-afc-orange-goalkeeper-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/sunderland-afc-green-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -3327,20 +3068,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-29 02:34</t>
+          <t>2026-10-29 02:29</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>85306</v>
+        <v>85295</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CFS_SAFC_YellowGK_KD_No_26/27</t>
+          <t>CFS_SAFC_OrangeGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sunderland AFC Yellow Goalkeeper Kids Cheap Football Kit 2026/27</t>
+          <t>Sunderland AFC Orange Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3366,7 +3107,7 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/sunderland-afc-yellow-goalkeeper-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/sunderland-afc-orange-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -3385,46 +3126,46 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-29 03:24</t>
+          <t>2026-10-29 02:34</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>85339</v>
+        <v>85306</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CFS_ATM_BlueTN_ADK_No_25/26</t>
+          <t>CFS_SAFC_YellowGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Atletico Madrid Blue Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Sunderland AFC Yellow Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
+          <t>Chưa có dữ liệu Sunderland đá giải nào mùa 2026/27 → cần người check option badge.</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/atletico-madrid-blue-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/sunderland-afc-yellow-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -3461,22 +3202,22 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -3501,46 +3242,46 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-29 03:34</t>
+          <t>2026-10-29 03:24</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>85346</v>
+        <v>85339</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CFS_ATM_PurpleTN_ADK_No_25/26</t>
+          <t>CFS_ATM_BlueTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Atletico Madrid Purple Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Atletico Madrid Blue Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/atletico-madrid-purple-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/atletico-madrid-blue-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -3577,22 +3318,22 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -3617,46 +3358,46 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-29 03:57</t>
+          <t>2026-10-29 03:34</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>85353</v>
+        <v>85346</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CFS_BM_GreenTN_ADK_No_25/26</t>
+          <t>CFS_ATM_PurpleTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bayern Munich Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Atletico Madrid Purple Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 71 ký tự (nên &lt;= 60)</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/bayern-munich-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/atletico-madrid-purple-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -3693,22 +3434,22 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Bayern Munich (Adidas): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>SEO title dài 71 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -3751,22 +3492,22 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>Club bị report</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>Ảnh</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Số lượng ảnh</t>
-        </is>
-      </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Bayern Munich (Adidas): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -3791,46 +3532,46 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-29 09:32</t>
+          <t>2026-10-29 03:57</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>85385</v>
+        <v>85353</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CFS_BM_OrangeTN_ADK_No_25/26</t>
+          <t>CFS_BM_GreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Bayern Munich Orange Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Bayern Munich Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/bayern-munich-orange-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -3867,22 +3608,22 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Bayern Munich (Adidas): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -3925,22 +3666,22 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>Club bị report</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
           <t>Ảnh</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Số lượng ảnh</t>
-        </is>
-      </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Bayern Munich (Adidas): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -3965,46 +3706,46 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-29 09:36</t>
+          <t>2026-10-29 09:32</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>85392</v>
+        <v>85385</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CFS_CHE_GreenTN_ADK_No_25/26</t>
+          <t>CFS_BM_OrangeTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Chelsea Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Bayern Munich Orange Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Chelsea (Nike): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-orange-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -4041,22 +3782,22 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>Club bị report</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
           <t>Ảnh</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Số lượng ảnh</t>
-        </is>
-      </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chelsea (Nike): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -4081,46 +3822,46 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-29 09:42</t>
+          <t>2026-10-29 09:36</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>85400</v>
+        <v>85392</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
+          <t>CFS_CHE_GreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
+          <t>Chelsea Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Chelsea (Nike): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -4157,22 +3898,22 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
+          <t>Club bị report</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
           <t>Ảnh</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Số lượng ảnh</t>
-        </is>
-      </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chelsea (Nike): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -4197,20 +3938,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-29 09:47</t>
+          <t>2026-10-29 09:42</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>85408</v>
+        <v>85400</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CFS_INM_BlackTN_ADK_No_25/26</t>
+          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Inter Miami Black Training Adult Cheap Football Kit 2025/26</t>
+          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4236,7 +3977,7 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-miami-black-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr">
@@ -4273,22 +4014,22 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Inter Miami có badge vô địch MLS nhưng LA Galaxy mới là nhà vô địch 2024 → cần người check.</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -4313,46 +4054,46 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-29 09:56</t>
+          <t>2026-10-29 09:47</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>85416</v>
+        <v>85408</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CFS_INM_WhiteTN_ADK_No_25/26</t>
+          <t>CFS_INM_BlackTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Inter Miami White Training Adult Cheap Football Kit 2025/26</t>
+          <t>Inter Miami Black Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Inter Miami có badge vô địch MLS nhưng LA Galaxy mới là nhà vô địch 2024 → cần người check.</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-miami-white-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/inter-miami-black-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
@@ -4389,22 +4130,22 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>Inter Miami có badge vô địch MLS nhưng LA Galaxy mới là nhà vô địch 2024 → cần người check.</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
@@ -4429,46 +4170,46 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-29 13:15</t>
+          <t>2026-10-29 09:56</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>85436</v>
+        <v>85416</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CFS_LV_BlackTN_ADK_No_25/26</t>
+          <t>CFS_INM_WhiteTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Liverpool Black Training Adult Cheap Football Kit 2025/26</t>
+          <t>Inter Miami White Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Inter Miami có badge vô địch MLS nhưng LA Galaxy mới là nhà vô địch 2024 → cần người check.</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/liverpool-black-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/inter-miami-white-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr">
@@ -4487,20 +4228,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-10-29 13:22</t>
+          <t>2026-10-29 13:15</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>85444</v>
+        <v>85436</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CFS_LV_WhiteTN_ADK_No_25/26</t>
+          <t>CFS_LV_BlackTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Liverpool White Training Adult Cheap Football Kit 2025/26</t>
+          <t>Liverpool Black Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4526,7 +4267,7 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/liverpool-white-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/liverpool-black-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
@@ -4545,20 +4286,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-29 14:20</t>
+          <t>2026-10-29 13:22</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>85519</v>
+        <v>85444</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CFS_RM_BlackTN_ADK_No_25/26</t>
+          <t>CFS_LV_WhiteTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Real Madrid Black Training Adult Cheap Football Kit 2025/26</t>
+          <t>Liverpool White Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4584,7 +4325,7 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-black-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/liverpool-white-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr">
@@ -4603,20 +4344,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-10-29 14:30</t>
+          <t>2026-10-29 14:20</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>85528</v>
+        <v>85519</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CFS_RM_BlueTN_ADK_No_25/26</t>
+          <t>CFS_RM_BlackTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Real Madrid Blue Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Black Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4642,7 +4383,7 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-blue-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-black-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr">
@@ -4661,20 +4402,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-10-29 14:35</t>
+          <t>2026-10-29 14:30</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>85536</v>
+        <v>85528</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CFS_RM_GreyTN_ADK_No_25/26</t>
+          <t>CFS_RM_BlueTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Real Madrid Grey Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Blue Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4700,7 +4441,7 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-grey-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-blue-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr">
@@ -4719,20 +4460,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-10-29 14:45</t>
+          <t>2026-10-29 14:35</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>85544</v>
+        <v>85536</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CFS_RM_HO_ADK_No_25/26</t>
+          <t>CFS_RM_GreyTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Real Madrid Home Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Grey Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4747,7 +4488,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -4758,7 +4499,7 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-home-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-grey-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr">
@@ -4777,20 +4518,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-10-29 14:50</t>
+          <t>2026-10-29 14:45</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>85552</v>
+        <v>85544</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CFS_RM_WhiteTN_ADK_No_25/26</t>
+          <t>CFS_RM_HO_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Real Madrid White Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Home Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4816,7 +4557,7 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-white-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-home-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr">
@@ -4835,20 +4576,20 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-10-29 14:53</t>
+          <t>2026-10-29 14:50</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>85560</v>
+        <v>85552</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CFS_RM_YellowTN_ADK_No_25/26</t>
+          <t>CFS_RM_WhiteTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Real Madrid Yellow Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid White Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4863,7 +4604,7 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -4874,7 +4615,7 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-yellow-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-white-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr">
@@ -4886,57 +4627,53 @@
       <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-10-29 03:24</t>
+          <t>2026-10-29 14:53</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>85339</v>
+        <v>85560</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>CFS_ATM_BlueTN_ADK_No_25/26</t>
+          <t>CFS_RM_YellowTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Atletico Madrid Blue Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Yellow Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sai season</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Tên sản phẩm</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Thêm ảnh</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/atletico-madrid-blue-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-yellow-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr">
@@ -4947,938 +4684,8 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>2026-10-29 03:34</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>85346</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>CFS_ATM_PurpleTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Atletico Madrid Purple Pre Match Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I43" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/atletico-madrid-purple-pre-match-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L43" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>2026-10-29 03:57</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>85353</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>CFS_BM_GreenTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Bayern Munich Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/bayern-munich-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L44" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2026-10-29 09:32</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>85385</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>CFS_BM_OrangeTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Bayern Munich Orange Pre Match Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I45" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/bayern-munich-orange-pre-match-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L45" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>2026-10-29 09:36</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>85392</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>CFS_CHE_GreenTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Chelsea Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I46" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L46" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2026-10-29 09:42</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>85400</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I47" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L47" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>2026-10-29 09:47</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>85408</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>CFS_INM_BlackTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Inter Miami Black Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/inter-miami-black-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L48" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>2026-10-29 09:56</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>85416</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>CFS_INM_WhiteTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Inter Miami White Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/inter-miami-white-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L49" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>2026-10-29 13:15</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>85436</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>CFS_LV_BlackTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Liverpool Black Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H50" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I50" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/liverpool-black-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L50" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>2026-10-29 13:22</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>85444</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>CFS_LV_WhiteTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Liverpool White Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/liverpool-white-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L51" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>2026-10-29 14:20</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>85519</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>CFS_RM_BlackTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Real Madrid Black Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H52" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I52" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-black-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L52" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>2026-10-29 14:30</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>85528</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>CFS_RM_BlueTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Real Madrid Blue Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H53" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I53" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-blue-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L53" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>2026-10-29 14:35</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>85536</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>CFS_RM_GreyTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Real Madrid Grey Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I54" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-grey-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L54" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>2026-10-29 14:45</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>85544</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>CFS_RM_HO_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Real Madrid Home Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H55" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I55" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-home-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L55" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>2026-10-29 14:50</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>85552</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>CFS_RM_WhiteTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Real Madrid White Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H56" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I56" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-white-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L56" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>2026-10-29 14:53</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>85560</v>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>CFS_RM_YellowTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Real Madrid Yellow Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Sai season</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm</t>
-        </is>
-      </c>
-      <c r="H57" s="5" t="inlineStr">
-        <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
-        </is>
-      </c>
-      <c r="I57" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-yellow-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L57" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N57"/>
+  <autoFilter ref="A1:N42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -5962,36 +4769,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId112"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Badge template line not a word to avoid; Free Pin promo check removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149ELLgZdjaY7wRsdGLp26m
</commit_message>
<xml_diff>
--- a/listing-monitor/reports/2026-10-29/qa_2026-10-29.xlsx
+++ b/listing-monitor/reports/2026-10-29/qa_2026-10-29.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cần xác nhận" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'KFK'!$A$1:$N$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CFS'!$A$1:$N$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'KFK'!$A$1:$N$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CFS'!$A$1:$N$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tạo lúc 2026-10-30 06:55. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
+          <t>Tạo lúc 2026-10-30 07:05. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
         <v>14</v>
@@ -565,7 +565,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G6" t="n">
         <v>31</v>
@@ -606,176 +606,144 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Khuyến mãi Free Pin (KFK)</t>
+          <t>Màu</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Màu</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="C11" t="n">
-        <v>1</v>
-      </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Sai season</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sai season</t>
+          <t>Sai đối tượng</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sai đối tượng</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Sai cầu thủ</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>4</v>
-      </c>
-      <c r="C19" t="n">
-        <v>4</v>
-      </c>
-      <c r="D19" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Sai cầu thủ</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -790,7 +758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -889,46 +857,46 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 09:12</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>265823</v>
+        <v>265852</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_ARG_AWLV_KD_No_1994</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Khuyến mãi Free Pin (KFK)</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Trang sản phẩm</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Sản phẩm Argentina (1 trong 7 đội có Free Pin) nhưng trang không có chữ 'FREE ARGENTINA PIN'</t>
+          <t>1/5 ảnh không có alt text</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra BOGO coupon buy-argentina-get-pin có gồm sản phẩm này không</t>
+          <t>Thêm alt text riêng cho từng ảnh</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -947,46 +915,46 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 15:48</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>265840</v>
+        <v>265918</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
+          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Khuyến mãi Free Pin (KFK)</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Trang sản phẩm</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Sản phẩm Argentina (1 trong 7 đội có Free Pin) nhưng trang không có chữ 'FREE ARGENTINA PIN'</t>
+          <t>1/7 ảnh không có alt text</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra BOGO coupon buy-argentina-get-pin có gồm sản phẩm này không</t>
+          <t>Thêm alt text riêng cho từng ảnh</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -1005,46 +973,46 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-29 09:12</t>
+          <t>2026-10-29 15:48</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>265852</v>
+        <v>265918</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_No_1994</t>
+          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 (No Socks, Long Sleeve)</t>
+          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Alt text</t>
+          <t>SKU variation</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>1/5 ảnh không có alt text</t>
+          <t>SKU cha KFK_CH_HO/AWGP_ADK_No_26/27 nhưng variation mang SKU khác đầu: KFK_CH_AW/HOGP_ADK_No_26/27_S (+4)</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Thêm alt text riêng cho từng ảnh</t>
+          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -1056,53 +1024,53 @@
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-29 09:12</t>
+          <t>2026-10-29 08:35</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>265852</v>
+        <v>265823</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_No_1994</t>
+          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 (No Socks, Long Sleeve)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Khuyến mãi Free Pin (KFK)</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Trang sản phẩm</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Sản phẩm Argentina (1 trong 7 đội có Free Pin) nhưng trang không có chữ 'FREE ARGENTINA PIN'</t>
+          <t>SEO title dài 70 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra BOGO coupon buy-argentina-get-pin có gồm sản phẩm này không</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -1114,53 +1082,53 @@
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-29 15:34</t>
+          <t>2026-10-29 08:35</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>265903</v>
+        <v>265823</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
+          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Meta description</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>'Badge' (...p to 13 letters and 2 digits. Badge options: Premier League sleev...)</t>
+          <t>Meta dài 169 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Badge -&gt; chest detail</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -1172,53 +1140,53 @@
       <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-29 15:48</t>
+          <t>2026-10-29 08:35</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>265918</v>
+        <v>265823</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
+          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>'badge' (...to 2 digits. Adult’s Home kit badge options: Premier League sleev...)</t>
+          <t>Alt text bị trùng giữa các ảnh: "Argentina Away Kids Kit 1994-MARADONA 10-over view-long sleeve-no socks"</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>badge -&gt; chest detail</t>
+          <t>Mỗi ảnh 1 alt riêng</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -1230,53 +1198,53 @@
       <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-29 15:48</t>
+          <t>2026-10-29 08:35</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>265918</v>
+        <v>265823</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
+          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Alt text</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>1/7 ảnh không có alt text</t>
+          <t>SKU 'KFK_ARG_AWLV_KD_MESSI 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Thêm alt text riêng cho từng ảnh</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -1288,53 +1256,53 @@
       <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-29 15:48</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>265918</v>
+        <v>265834</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
+          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
+          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Sai cầu thủ</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SKU variation</t>
+          <t>Tên sản phẩm</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>SKU cha KFK_CH_HO/AWGP_ADK_No_26/27 nhưng variation mang SKU khác đầu: KFK_CH_AW/HOGP_ADK_No_26/27_S (+4)</t>
+          <t>Tên + số cầu thủ chưa VIẾT HOA</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
+          <t>Viết hoa tên + số cầu thủ</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1353,20 +1321,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>265823</v>
+        <v>265834</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1381,7 +1349,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 70 ký tự (nên &lt;= 60)</t>
+          <t>SEO title dài 66 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1392,7 +1360,7 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1411,46 +1379,46 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>265823</v>
+        <v>265834</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Meta description</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 169 ký tự (nên &lt;= 160)</t>
+          <t>Alt text bị trùng giữa các ảnh: "Inter Milan Home kids kit 2009_10-IBRAHIMOVIĆ 8-back view-no socks"</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Mỗi ảnh 1 alt riêng</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1469,46 +1437,46 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>265823</v>
+        <v>265834</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Alt text</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Alt text bị trùng giữa các ảnh: "Argentina Away Kids Kit 1994-MARADONA 10-over view-long sleeve-no socks"</t>
+          <t>SKU 'KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Mỗi ảnh 1 alt riêng</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1527,46 +1495,46 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-29 08:35</t>
+          <t>2026-10-29 08:51</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>265823</v>
+        <v>265840</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MESSI 10 (No Socks, Long Sleeve)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>SKU 'KFK_ARG_AWLV_KD_MESSI 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SEO title dài 73 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-messi-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -1589,42 +1557,42 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>265834</v>
+        <v>265840</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
+          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Sai cầu thủ</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Tên sản phẩm</t>
+          <t>Meta description</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Tên + số cầu thủ chưa VIẾT HOA</t>
+          <t>Meta dài 172 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Viết hoa tên + số cầu thủ</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1647,42 +1615,42 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>265834</v>
+        <v>265840</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
+          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
+          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 66 ký tự (nên &lt;= 60)</t>
+          <t>SKU 'KFK_ARG_AWLV_KD_MARADONA 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
+          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -1701,46 +1669,46 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 15:34</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>265834</v>
+        <v>265903</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
+          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
+          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Alt text</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Alt text bị trùng giữa các ảnh: "Inter Milan Home kids kit 2009_10-IBRAHIMOVIĆ 8-back view-no socks"</t>
+          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Mỗi ảnh 1 alt riêng</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -1759,46 +1727,46 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 15:34</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>265834</v>
+        <v>265903</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10</t>
+          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Retro Inter Milan Home Kids Football Kit 2009/10 – IBRAHIMOVIĆ 8 (No Socks)</t>
+          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>SKU 'KFK_IM_HO_KD_IBRAHIMOVIĆ 8_09/10' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Chelsea (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-inter-milan-home-kids-football-kit-2009-10-ibrahimovic-8/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1817,46 +1785,46 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-29 08:51</t>
+          <t>2026-10-29 15:48</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>265840</v>
+        <v>265918</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
+          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 73 ký tự (nên &lt;= 60)</t>
+          <t>Chelsea (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
+          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1867,298 +1835,8 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-10-29 08:51</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>265840</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Meta description</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>Meta dài 172 ký tự (nên &lt;= 160)</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>Rút gọn</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-10-29 08:51</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>265840</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>KFK_ARG_AWLV_KD_MARADONA 10_1994</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Retro Argentina Away Kids Football Kit 1994 – MARADONA 10 (No Socks, Long Sleeve)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>SKU (Google)</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>SKU 'KFK_ARG_AWLV_KD_MARADONA 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>https://kidsfootballkit.co.uk/product/retro-argentina-away-kids-football-kit-1994-maradona-10-long-sleeve/</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2026-10-29 15:34</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>265903</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>SEO title</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>Rút gọn</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
-        </is>
-      </c>
-      <c r="L21" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2026-10-29 15:34</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>265903</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>KFK_CH_OrangeGK_ADK_No_26/27</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Chelsea Goalkeeper Adult Football Kit 2026/27 (No Socks) – Orange</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Club bị report</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>Chelsea (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>Check blur logo</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-goalkeeper-adult-football-kit-2026-27-orange/</t>
-        </is>
-      </c>
-      <c r="L22" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-10-29 15:48</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>265918</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>KFK_CH_HO/AWGP_ADK_No_26/27</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Chelsea Gift Pack – Home and Away Adult Football Kit 2026/27 (With socks)</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Club bị report</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Chelsea (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>Check blur logo</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>https://kidsfootballkit.co.uk/product/chelsea-gift-pack-home-and-away-adult-football-kit-2026-27/</t>
-        </is>
-      </c>
-      <c r="L23" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N23"/>
+  <autoFilter ref="A1:N18"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -2194,16 +1872,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2215,7 +1883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2622,22 +2290,22 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>'badge' (... letters and 2 digits. Sleeve badge: Combo Chelsea 2025 badge can...)</t>
+          <t>Option "Add Combo Chelsea Badge 2025" không ghi tên giải (ảnh/gợi ý: Premier League).</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>badge -&gt; chest detail</t>
+          <t>Ghi tên giải vào tên option (vd 'Add Premier League Badge')</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -2662,20 +2330,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-29 09:36</t>
+          <t>2026-10-29 09:42</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>85392</v>
+        <v>85400</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CFS_CHE_GreenTN_ADK_No_25/26</t>
+          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Chelsea Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2701,7 +2369,7 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -2720,46 +2388,46 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-29 09:42</t>
+          <t>2026-10-29 14:45</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>85400</v>
+        <v>85544</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
+          <t>CFS_RM_HO_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Home Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Sai season</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Tên sản phẩm</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>'badge' (... letters and 2 digits. Sleeve badge: Combo Chelsea 2025 badge can...)</t>
+          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>badge -&gt; chest detail</t>
+          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-home-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -2771,53 +2439,53 @@
       <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-29 09:42</t>
+          <t>2026-10-29 01:43</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>85400</v>
+        <v>85240</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
+          <t>CFS_MC_HOLV_KD_No_26/27</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
+          <t>Manchester City Home Kids Cheap Football Kit 2026/27 Long Sleeve</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Option "Add Combo Chelsea Badge 2025" không ghi tên giải (ảnh/gợi ý: Premier League).</t>
+          <t>Manchester City (Puma): sheet ghi CFS 'Published (blurred PUMA logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Ghi tên giải vào tên option (vd 'Add Premier League Badge')</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/manchester-city-home-kids-cheap-football-kit-2026-27-long-sleeve/</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -2829,53 +2497,53 @@
       <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-29 14:45</t>
+          <t>2026-10-29 02:00</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>85544</v>
+        <v>85273</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CFS_RM_HO_ADK_No_25/26</t>
+          <t>CFS_SHW_AW_KD_No_26/27</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Real Madrid Home Adult Cheap Football Kit 2025/26</t>
+          <t>Sheffield Wednesday Away Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sai season</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Tên sản phẩm</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Listing mới nhưng season là 25/26, không phải 26/27</t>
+          <t>Không xác định được đội/CLB từ tên sản phẩm → cần người check option badge.</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra lại season (club: 26/27, đội tuyển: 2026, retro: giữ nguyên)</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-home-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/sheffield-wednesday-away-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -2894,46 +2562,46 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-29 01:43</t>
+          <t>2026-10-29 02:06</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>85240</v>
+        <v>85284</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CFS_MC_HOLV_KD_No_26/27</t>
+          <t>CFS_SAFC_GreenGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Manchester City Home Kids Cheap Football Kit 2026/27 Long Sleeve</t>
+          <t>Sunderland AFC Green Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Manchester City (Puma): sheet ghi CFS 'Published (blurred PUMA logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Chưa có dữ liệu Sunderland đá giải nào mùa 2026/27 → cần người check option badge.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/manchester-city-home-kids-cheap-football-kit-2026-27-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/sunderland-afc-green-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -2952,20 +2620,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-29 02:00</t>
+          <t>2026-10-29 02:29</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>85273</v>
+        <v>85295</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CFS_SHW_AW_KD_No_26/27</t>
+          <t>CFS_SAFC_OrangeGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sheffield Wednesday Away Kids Cheap Football Kit 2026/27</t>
+          <t>Sunderland AFC Orange Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2980,7 +2648,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Không xác định được đội/CLB từ tên sản phẩm → cần người check option badge.</t>
+          <t>Chưa có dữ liệu Sunderland đá giải nào mùa 2026/27 → cần người check option badge.</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -2991,7 +2659,7 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/sheffield-wednesday-away-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/sunderland-afc-orange-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -3010,20 +2678,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-29 02:06</t>
+          <t>2026-10-29 02:34</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>85284</v>
+        <v>85306</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CFS_SAFC_GreenGK_KD_No_26/27</t>
+          <t>CFS_SAFC_YellowGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sunderland AFC Green Goalkeeper Kids Cheap Football Kit 2026/27</t>
+          <t>Sunderland AFC Yellow Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3049,7 +2717,7 @@
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/sunderland-afc-green-goalkeeper-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/sunderland-afc-yellow-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -3068,46 +2736,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-29 02:29</t>
+          <t>2026-10-29 03:24</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>85295</v>
+        <v>85339</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CFS_SAFC_OrangeGK_KD_No_26/27</t>
+          <t>CFS_ATM_BlueTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sunderland AFC Orange Goalkeeper Kids Cheap Football Kit 2026/27</t>
+          <t>Atletico Madrid Blue Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu Sunderland đá giải nào mùa 2026/27 → cần người check option badge.</t>
+          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/sunderland-afc-orange-goalkeeper-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/atletico-madrid-blue-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -3126,46 +2794,46 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-29 02:34</t>
+          <t>2026-10-29 03:24</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>85306</v>
+        <v>85339</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CFS_SAFC_YellowGK_KD_No_26/27</t>
+          <t>CFS_ATM_BlueTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sunderland AFC Yellow Goalkeeper Kids Cheap Football Kit 2026/27</t>
+          <t>Atletico Madrid Blue Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu Sunderland đá giải nào mùa 2026/27 → cần người check option badge.</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/sunderland-afc-yellow-goalkeeper-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/atletico-madrid-blue-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -3184,20 +2852,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-29 03:24</t>
+          <t>2026-10-29 03:34</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>85339</v>
+        <v>85346</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CFS_ATM_BlueTN_ADK_No_25/26</t>
+          <t>CFS_ATM_PurpleTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Atletico Madrid Blue Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Atletico Madrid Purple Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3212,7 +2880,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
+          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -3223,7 +2891,7 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/atletico-madrid-blue-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/atletico-madrid-purple-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -3242,20 +2910,20 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-29 03:24</t>
+          <t>2026-10-29 03:34</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>85339</v>
+        <v>85346</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CFS_ATM_BlueTN_ADK_No_25/26</t>
+          <t>CFS_ATM_PurpleTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Atletico Madrid Blue Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Atletico Madrid Purple Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3281,7 +2949,7 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/atletico-madrid-blue-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/atletico-madrid-purple-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -3300,20 +2968,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-29 03:34</t>
+          <t>2026-10-29 03:57</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>85346</v>
+        <v>85353</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CFS_ATM_PurpleTN_ADK_No_25/26</t>
+          <t>CFS_BM_GreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Atletico Madrid Purple Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Bayern Munich Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3328,7 +2996,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
+          <t>SEO title dài 71 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -3339,7 +3007,7 @@
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/atletico-madrid-purple-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -3358,46 +3026,46 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-29 03:34</t>
+          <t>2026-10-29 03:57</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>85346</v>
+        <v>85353</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CFS_ATM_PurpleTN_ADK_No_25/26</t>
+          <t>CFS_BM_GreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Atletico Madrid Purple Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Bayern Munich Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>Club bị report</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>Ảnh</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Số lượng ảnh</t>
-        </is>
-      </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Bayern Munich (Adidas): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/atletico-madrid-purple-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -3434,22 +3102,22 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 71 ký tự (nên &lt;= 60)</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -3474,46 +3142,46 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-29 03:57</t>
+          <t>2026-10-29 09:32</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>85353</v>
+        <v>85385</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CFS_BM_GreenTN_ADK_No_25/26</t>
+          <t>CFS_BM_OrangeTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bayern Munich Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Bayern Munich Orange Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Bayern Munich (Adidas): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/bayern-munich-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-orange-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -3532,46 +3200,46 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-29 03:57</t>
+          <t>2026-10-29 09:32</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>85353</v>
+        <v>85385</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CFS_BM_GreenTN_ADK_No_25/26</t>
+          <t>CFS_BM_OrangeTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Bayern Munich Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Bayern Munich Orange Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>Club bị report</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
           <t>Ảnh</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Số lượng ảnh</t>
-        </is>
-      </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Bayern Munich (Adidas): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/bayern-munich-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-orange-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -3608,22 +3276,22 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -3648,20 +3316,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-29 09:32</t>
+          <t>2026-10-29 09:36</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>85385</v>
+        <v>85392</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CFS_BM_OrangeTN_ADK_No_25/26</t>
+          <t>CFS_CHE_GreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Bayern Munich Orange Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Chelsea Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3676,7 +3344,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Bayern Munich (Adidas): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Chelsea (Nike): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -3687,7 +3355,7 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/bayern-munich-orange-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -3706,20 +3374,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-29 09:32</t>
+          <t>2026-10-29 09:36</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>85385</v>
+        <v>85392</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CFS_BM_OrangeTN_ADK_No_25/26</t>
+          <t>CFS_CHE_GreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bayern Munich Orange Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Chelsea Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3745,7 +3413,7 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/bayern-munich-orange-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -3764,20 +3432,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-29 09:36</t>
+          <t>2026-10-29 09:42</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>85392</v>
+        <v>85400</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CFS_CHE_GreenTN_ADK_No_25/26</t>
+          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Chelsea Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3803,7 +3471,7 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -3822,20 +3490,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-29 09:36</t>
+          <t>2026-10-29 09:42</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>85392</v>
+        <v>85400</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CFS_CHE_GreenTN_ADK_No_25/26</t>
+          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Chelsea Green Pre Match Training Adult Cheap Football Kit 2025/26</t>
+          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3850,7 +3518,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -3861,7 +3529,7 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-green-pre-match-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -3880,46 +3548,46 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-29 09:42</t>
+          <t>2026-10-29 09:47</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>85400</v>
+        <v>85408</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
+          <t>CFS_INM_BlackTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
+          <t>Inter Miami Black Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Chelsea (Nike): sheet ghi CFS 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/inter-miami-black-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr">
@@ -3938,46 +3606,46 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-29 09:42</t>
+          <t>2026-10-29 09:47</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>85400</v>
+        <v>85408</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CFS_CHE_LightGreenTN_ADK_No_25/26</t>
+          <t>CFS_INM_BlackTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Chelsea Light Green Training Adult Cheap Football Kit 2025/26</t>
+          <t>Inter Miami Black Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Inter Miami có badge vô địch MLS nhưng LA Galaxy mới là nhà vô địch 2024 → cần người check.</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-light-green-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/inter-miami-black-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr">
@@ -3996,20 +3664,20 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-10-29 09:47</t>
+          <t>2026-10-29 09:56</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>85408</v>
+        <v>85416</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CFS_INM_BlackTN_ADK_No_25/26</t>
+          <t>CFS_INM_WhiteTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Inter Miami Black Training Adult Cheap Football Kit 2025/26</t>
+          <t>Inter Miami White Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4035,7 +3703,7 @@
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-miami-black-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/inter-miami-white-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr">
@@ -4054,20 +3722,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-29 09:47</t>
+          <t>2026-10-29 09:56</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>85408</v>
+        <v>85416</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CFS_INM_BlackTN_ADK_No_25/26</t>
+          <t>CFS_INM_WhiteTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Inter Miami Black Training Adult Cheap Football Kit 2025/26</t>
+          <t>Inter Miami White Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4093,7 +3761,7 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-miami-black-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/inter-miami-white-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
@@ -4112,20 +3780,20 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-10-29 09:56</t>
+          <t>2026-10-29 13:15</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>85416</v>
+        <v>85436</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CFS_INM_WhiteTN_ADK_No_25/26</t>
+          <t>CFS_LV_BlackTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Inter Miami White Training Adult Cheap Football Kit 2025/26</t>
+          <t>Liverpool Black Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4151,7 +3819,7 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-miami-white-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/liverpool-black-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr">
@@ -4170,46 +3838,46 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-29 09:56</t>
+          <t>2026-10-29 13:22</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>85416</v>
+        <v>85444</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CFS_INM_WhiteTN_ADK_No_25/26</t>
+          <t>CFS_LV_WhiteTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Inter Miami White Training Adult Cheap Football Kit 2025/26</t>
+          <t>Liverpool White Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Inter Miami có badge vô địch MLS nhưng LA Galaxy mới là nhà vô địch 2024 → cần người check.</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-miami-white-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/liverpool-white-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr">
@@ -4228,20 +3896,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-10-29 13:15</t>
+          <t>2026-10-29 14:20</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>85436</v>
+        <v>85519</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CFS_LV_BlackTN_ADK_No_25/26</t>
+          <t>CFS_RM_BlackTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Liverpool Black Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Black Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4267,7 +3935,7 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/liverpool-black-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-black-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
@@ -4286,20 +3954,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-29 13:22</t>
+          <t>2026-10-29 14:30</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>85444</v>
+        <v>85528</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CFS_LV_WhiteTN_ADK_No_25/26</t>
+          <t>CFS_RM_BlueTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Liverpool White Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Blue Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4325,7 +3993,7 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/liverpool-white-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-blue-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr">
@@ -4344,20 +4012,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-10-29 14:20</t>
+          <t>2026-10-29 14:35</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>85519</v>
+        <v>85536</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CFS_RM_BlackTN_ADK_No_25/26</t>
+          <t>CFS_RM_GreyTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Real Madrid Black Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Grey Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4383,7 +4051,7 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-black-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-grey-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr">
@@ -4402,20 +4070,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-10-29 14:30</t>
+          <t>2026-10-29 14:45</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>85528</v>
+        <v>85544</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CFS_RM_BlueTN_ADK_No_25/26</t>
+          <t>CFS_RM_HO_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Real Madrid Blue Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Home Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4430,7 +4098,7 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
@@ -4441,7 +4109,7 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-blue-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-home-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr">
@@ -4460,20 +4128,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-10-29 14:35</t>
+          <t>2026-10-29 14:50</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>85536</v>
+        <v>85552</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CFS_RM_GreyTN_ADK_No_25/26</t>
+          <t>CFS_RM_WhiteTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Real Madrid Grey Training Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid White Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4488,7 +4156,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -4499,7 +4167,7 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-grey-training-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-white-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr">
@@ -4518,20 +4186,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-10-29 14:45</t>
+          <t>2026-10-29 14:53</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>85544</v>
+        <v>85560</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CFS_RM_HO_ADK_No_25/26</t>
+          <t>CFS_RM_YellowTN_ADK_No_25/26</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Real Madrid Home Adult Cheap Football Kit 2025/26</t>
+          <t>Real Madrid Yellow Training Adult Cheap Football Kit 2025/26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4546,7 +4214,7 @@
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
@@ -4557,7 +4225,7 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-home-adult-cheap-football-kit-2025-26/</t>
+          <t>https://cheapfootballshirts.com/product/real-madrid-yellow-training-adult-cheap-football-kit-2025-26/</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr">
@@ -4568,124 +4236,8 @@
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
     </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>2026-10-29 14:50</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>85552</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>CFS_RM_WhiteTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Real Madrid White Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Số lượng ảnh</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>Chỉ có 1 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>Thêm ảnh</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-white-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L41" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>2026-10-29 14:53</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>85560</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>CFS_RM_YellowTN_ADK_No_25/26</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Real Madrid Yellow Training Adult Cheap Football Kit 2025/26</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Số lượng ảnh</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>Thêm ảnh</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/real-madrid-yellow-training-adult-cheap-football-kit-2025-26/</t>
-        </is>
-      </c>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N42"/>
+  <autoFilter ref="A1:N40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -4765,10 +4317,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4780,7 +4328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4814,70 +4362,58 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Free Pin (KFK)</t>
+          <t>Tên né thương hiệu</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Tool cũ: 7 đội Spain/France/Argentina/England/Brazil/Portugal/Scotland phải có chữ 'FREE [TEAM] PIN' trên trang. Ngày 2/10 không tìm thấy chữ này trong HTML trang. Khuyến mãi còn chạy không?</t>
+          <t>Tool coi 'North London Red' = Arsenal, 'P^_^SG' = PSG và nhận ra kiểu 'Arsn@l', 'Lvr^_^pooI'.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tên né thương hiệu</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Tool coi 'North London Red' = Arsenal, 'P^_^SG' = PSG và nhận ra kiểu 'Arsn@l', 'Lvr^_^pooI'.</t>
+          <t>Tool KHÔNG báo lỗi chữ 'badge' trong dòng template 'Badge options: ...' / 'Sleeve badge: ...' (đã xác nhận 30/10), chỉ báo 'badge' ở chỗ khác (vd 'club badge').</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Độ dài SEO title</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Tool KHÔNG báo lỗi 'sleeve badge' (tên option), chỉ báo 'badge' đứng riêng.</t>
+          <t>Tool báo khi SEO title &gt; 65 ký tự và meta &gt; 165 ký tự (mức Thấp).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Độ dài SEO title</t>
+          <t>KFK / CFS / RFK template SEO</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Tool báo khi SEO title &gt; 65 ký tự và meta &gt; 165 ký tự (mức Thấp).</t>
+          <t>SOP chưa có template SEO title/meta cho KFK, CFS, RFK nên tool chưa check đúng mẫu cho các site này, chỉ check nội dung có khớp sản phẩm không.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KFK / CFS / RFK template SEO</t>
+          <t>Đã xác nhận 27/9</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>SOP chưa có template SEO title/meta cho KFK, CFS, RFK nên tool chưa check đúng mẫu cho các site này, chỉ check nội dung có khớp sản phẩm không.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Đã xác nhận 27/9</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>ADK = Adult Kit. Gift pack noindex là cố ý (không báo lỗi). Listing in 'CHAMPIONS 26 / WINNERS 26' không cần player attribute. Nhắc 'short sleeve' được, chỉ báo khi mâu thuẫn với Long Sleeve (tên/SKU/ảnh).</t>
         </is>

</xml_diff>